<commit_message>
product material bulk import updated
</commit_message>
<xml_diff>
--- a/public/demo-files/board-pre-production-demo-file.xlsx
+++ b/public/demo-files/board-pre-production-demo-file.xlsx
@@ -25,7 +25,7 @@
     <t xml:space="preserve">PRODUCT CODE</t>
   </si>
   <si>
-    <t xml:space="preserve">TYPE OF WOOD</t>
+    <t xml:space="preserve">Type of Board (Raw Board)</t>
   </si>
   <si>
     <t xml:space="preserve">MACHINE USED</t>
@@ -77,11 +77,12 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
@@ -97,6 +98,13 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="0"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -141,17 +149,21 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -172,7 +184,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:J75"/>
-  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.55078125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="1" style="0" width="24.45"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="28.34"/>
@@ -183,7 +195,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="9" style="0" width="23.76"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" s="2" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -211,12 +223,12 @@
       <c r="I1" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="0" t="s">
+      <c r="J1" s="2" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="1" t="n">
+      <c r="A2" s="3" t="n">
         <v>1002</v>
       </c>
       <c r="B2" s="0" t="s">
@@ -248,7 +260,7 @@
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="1" t="n">
+      <c r="A3" s="3" t="n">
         <v>1003</v>
       </c>
       <c r="B3" s="0" t="s">
@@ -280,220 +292,220 @@
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="1"/>
+      <c r="A4" s="3"/>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="1"/>
+      <c r="A5" s="3"/>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="1"/>
+      <c r="A6" s="3"/>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="1"/>
+      <c r="A7" s="3"/>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="1"/>
+      <c r="A8" s="3"/>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="1"/>
+      <c r="A9" s="3"/>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="1"/>
+      <c r="A10" s="3"/>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="1"/>
+      <c r="A11" s="3"/>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="1"/>
+      <c r="A12" s="3"/>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="1"/>
+      <c r="A13" s="3"/>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="1"/>
+      <c r="A14" s="3"/>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="1"/>
+      <c r="A15" s="3"/>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="1"/>
+      <c r="A16" s="3"/>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="1"/>
+      <c r="A17" s="3"/>
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="1"/>
+      <c r="A18" s="3"/>
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="1"/>
+      <c r="A19" s="3"/>
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="1"/>
+      <c r="A20" s="3"/>
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="1"/>
+      <c r="A21" s="3"/>
     </row>
     <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="1"/>
+      <c r="A22" s="3"/>
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="1"/>
+      <c r="A23" s="3"/>
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="1"/>
+      <c r="A24" s="3"/>
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="1"/>
+      <c r="A25" s="3"/>
     </row>
     <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="1"/>
+      <c r="A26" s="3"/>
     </row>
     <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="1"/>
+      <c r="A27" s="3"/>
     </row>
     <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="1"/>
+      <c r="A28" s="3"/>
     </row>
     <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="1"/>
+      <c r="A29" s="3"/>
     </row>
     <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="1"/>
+      <c r="A30" s="3"/>
     </row>
     <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="1"/>
+      <c r="A31" s="3"/>
     </row>
     <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="1"/>
+      <c r="A32" s="3"/>
     </row>
     <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="1"/>
+      <c r="A33" s="3"/>
     </row>
     <row r="34" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="1"/>
+      <c r="A34" s="3"/>
     </row>
     <row r="35" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="1"/>
+      <c r="A35" s="3"/>
     </row>
     <row r="36" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="1"/>
+      <c r="A36" s="3"/>
     </row>
     <row r="37" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="1"/>
+      <c r="A37" s="3"/>
     </row>
     <row r="38" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="1"/>
+      <c r="A38" s="3"/>
     </row>
     <row r="39" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="1"/>
+      <c r="A39" s="3"/>
     </row>
     <row r="40" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="1"/>
+      <c r="A40" s="3"/>
     </row>
     <row r="41" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="1"/>
+      <c r="A41" s="3"/>
     </row>
     <row r="42" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="1"/>
+      <c r="A42" s="3"/>
     </row>
     <row r="43" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="1"/>
+      <c r="A43" s="3"/>
     </row>
     <row r="44" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="1"/>
+      <c r="A44" s="3"/>
     </row>
     <row r="45" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="1"/>
+      <c r="A45" s="3"/>
     </row>
     <row r="46" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="1"/>
+      <c r="A46" s="3"/>
     </row>
     <row r="47" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="1"/>
+      <c r="A47" s="3"/>
     </row>
     <row r="48" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="1"/>
+      <c r="A48" s="3"/>
     </row>
     <row r="49" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="1"/>
+      <c r="A49" s="3"/>
     </row>
     <row r="50" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A50" s="1"/>
+      <c r="A50" s="3"/>
     </row>
     <row r="51" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="1"/>
+      <c r="A51" s="3"/>
     </row>
     <row r="52" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A52" s="1"/>
+      <c r="A52" s="3"/>
     </row>
     <row r="53" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A53" s="1"/>
+      <c r="A53" s="3"/>
     </row>
     <row r="54" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A54" s="1"/>
+      <c r="A54" s="3"/>
     </row>
     <row r="55" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A55" s="1"/>
+      <c r="A55" s="3"/>
     </row>
     <row r="56" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A56" s="1"/>
+      <c r="A56" s="3"/>
     </row>
     <row r="57" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A57" s="1"/>
+      <c r="A57" s="3"/>
     </row>
     <row r="58" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A58" s="1"/>
+      <c r="A58" s="3"/>
     </row>
     <row r="59" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A59" s="1"/>
+      <c r="A59" s="3"/>
     </row>
     <row r="60" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A60" s="1"/>
+      <c r="A60" s="3"/>
     </row>
     <row r="61" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A61" s="1"/>
+      <c r="A61" s="3"/>
     </row>
     <row r="62" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A62" s="1"/>
+      <c r="A62" s="3"/>
     </row>
     <row r="63" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A63" s="1"/>
+      <c r="A63" s="3"/>
     </row>
     <row r="64" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A64" s="1"/>
+      <c r="A64" s="3"/>
     </row>
     <row r="65" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A65" s="1"/>
+      <c r="A65" s="3"/>
     </row>
     <row r="66" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A66" s="1"/>
+      <c r="A66" s="3"/>
     </row>
     <row r="67" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A67" s="1"/>
+      <c r="A67" s="3"/>
     </row>
     <row r="68" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A68" s="1"/>
+      <c r="A68" s="3"/>
     </row>
     <row r="69" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A69" s="1"/>
+      <c r="A69" s="3"/>
     </row>
     <row r="70" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A70" s="1"/>
+      <c r="A70" s="3"/>
     </row>
     <row r="71" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A71" s="1"/>
+      <c r="A71" s="3"/>
     </row>
     <row r="72" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A72" s="1"/>
+      <c r="A72" s="3"/>
     </row>
     <row r="73" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A73" s="1"/>
+      <c r="A73" s="3"/>
     </row>
     <row r="74" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A74" s="1"/>
+      <c r="A74" s="3"/>
     </row>
     <row r="75" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A75" s="1"/>
+      <c r="A75" s="3"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>